<commit_message>
upload: input_flight_plan for 2025-11-05 (051125/Flight_Plan.xlsx)
</commit_message>
<xml_diff>
--- a/outputs/2025-11-05/inputs/input_flight_plan.xlsx
+++ b/outputs/2025-11-05/inputs/input_flight_plan.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Flight Operations\Crew Sched and BD Shared Folder\2025\November\Input Files\Mu sigma\051125\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Flight Operations\Crew Sched and BD Shared Folder\2025\November\Input Files\KTree\051125\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0B22665-8DA9-4E7E-8886-3F8D04587957}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
@@ -1122,9 +1122,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1162,7 +1162,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1268,7 +1268,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1410,7 +1410,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>

</xml_diff>